<commit_message>
fix: polish PMM public copy and downloadable resources
</commit_message>
<xml_diff>
--- a/assets/downloads/ehs-sil-pmm-dialogue.xlsx
+++ b/assets/downloads/ehs-sil-pmm-dialogue.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="R4c3b0a8932f3403e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话记录" sheetId="2" r:id="Re65b97991c7f49ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行动跟进" sheetId="3" r:id="Rea90f0571c5f4549"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="解释参考" sheetId="4" r:id="Rddf957b71bc44697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="Rd0c12a6c69dd4471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话记录" sheetId="2" r:id="R509ceadcc2874a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行动跟进" sheetId="3" r:id="R03cf384b734e411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="解释参考" sheetId="4" r:id="R0d1950bcfadf4856"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -302,7 +302,7 @@
         <x:v>PMM 渐进式激励管理</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
-        <x:v>脱敏改编通用模板</x:v>
+        <x:v>对话与行动通用模板</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="55" customHeight="1">
@@ -371,10 +371,10 @@
     </x:row>
     <x:row r="10" ht="55" customHeight="1">
       <x:c r="A10" s="6" t="str">
-        <x:v>原材料处理</x:v>
+        <x:v>使用建议</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>依据用户提供的程序和表格重新制作。未复制企业标识、原图、人员信息、内部文号、隐藏数据或原文件元数据。</x:v>
+        <x:v>结合企业程序和现场情境使用；如纳入企业制度，应完成内部审核。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="55" customHeight="1">
@@ -547,7 +547,7 @@
       </x:c>
       <x:c r="B13" s="8" t="str"/>
       <x:c r="C13" s="7" t="str">
-        <x:v>分享前脱敏；按企业规则控制访问和留存</x:v>
+        <x:v>分享前检查并移除个人或保密信息；按企业规则控制访问和留存</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">

</xml_diff>

<commit_message>
fix: polish PMM public copy and downloadable resources (#28)
Co-authored-by: EHS-SIL <ehs-sil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/downloads/ehs-sil-pmm-dialogue.xlsx
+++ b/assets/downloads/ehs-sil-pmm-dialogue.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="R4c3b0a8932f3403e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话记录" sheetId="2" r:id="Re65b97991c7f49ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行动跟进" sheetId="3" r:id="Rea90f0571c5f4549"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="解释参考" sheetId="4" r:id="Rddf957b71bc44697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="Rd0c12a6c69dd4471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话记录" sheetId="2" r:id="R509ceadcc2874a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行动跟进" sheetId="3" r:id="R03cf384b734e411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="解释参考" sheetId="4" r:id="R0d1950bcfadf4856"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -302,7 +302,7 @@
         <x:v>PMM 渐进式激励管理</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
-        <x:v>脱敏改编通用模板</x:v>
+        <x:v>对话与行动通用模板</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="55" customHeight="1">
@@ -371,10 +371,10 @@
     </x:row>
     <x:row r="10" ht="55" customHeight="1">
       <x:c r="A10" s="6" t="str">
-        <x:v>原材料处理</x:v>
+        <x:v>使用建议</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>依据用户提供的程序和表格重新制作。未复制企业标识、原图、人员信息、内部文号、隐藏数据或原文件元数据。</x:v>
+        <x:v>结合企业程序和现场情境使用；如纳入企业制度，应完成内部审核。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="55" customHeight="1">
@@ -547,7 +547,7 @@
       </x:c>
       <x:c r="B13" s="8" t="str"/>
       <x:c r="C13" s="7" t="str">
-        <x:v>分享前脱敏；按企业规则控制访问和留存</x:v>
+        <x:v>分享前检查并移除个人或保密信息；按企业规则控制访问和留存</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">

</xml_diff>